<commit_message>
Simplify quiz flow: drop open-registration and next-question steps
Admin now only controls start/end; there's no separate registration-open
gate or per-question pacing. Participants can join a session's URL and
register any time before it ends, then get all 5 questions at once when
the admin starts the quiz and answer them self-paced. Ending the quiz
sends everyone straight to a results screen (leaderboard + AI analysis).

QuizSession status collapses to draft -> in_progress -> ended (drops
currentQuestionIndex and registration_open). GET /api/questions/:sessionId
now returns the full question set instead of a single "current" one, and
the questions:all socket event replaces the old per-question question:new
push. Updated README and the frontend build prompt/API spreadsheet to
match.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/MACROPAGE-Quiz-API-Endpoints.xlsx
+++ b/docs/MACROPAGE-Quiz-API-Endpoints.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="105">
   <si>
     <t>Group</t>
   </si>
@@ -87,40 +87,22 @@
     <t>{ title: string, autoSeedQuestions?: boolean (default true) }</t>
   </si>
   <si>
-    <t>QuizSession document (includes _id, status: "draft", currentQuestionIndex: -1, questionIds: [])</t>
-  </si>
-  <si>
-    <t>Creates a session; auto-seeds the 5 default questions unless autoSeedQuestions is false.</t>
-  </si>
-  <si>
-    <t>/api/sessions/:id/open-registration</t>
+    <t>QuizSession document (_id, status: "draft", questionIds: [])</t>
+  </si>
+  <si>
+    <t>Creates a session; auto-seeds the 5 default questions unless autoSeedQuestions is false. Registration is open immediately — no separate open-registration step.</t>
+  </si>
+  <si>
+    <t>/api/sessions/:id/start</t>
   </si>
   <si>
     <t>(none)</t>
   </si>
   <si>
-    <t>Updated QuizSession (status: "registration_open")</t>
-  </si>
-  <si>
-    <t>Only valid from status "draft". Broadcasts session:state over socket.</t>
-  </si>
-  <si>
-    <t>/api/sessions/:id/start</t>
-  </si>
-  <si>
-    <t>Updated QuizSession (status: "in_progress", currentQuestionIndex: 0)</t>
-  </si>
-  <si>
-    <t>Only valid from "registration_open" and requires questions configured. Broadcasts session:state + question:new.</t>
-  </si>
-  <si>
-    <t>/api/sessions/:id/next-question</t>
-  </si>
-  <si>
-    <t>Updated QuizSession (currentQuestionIndex incremented)</t>
-  </si>
-  <si>
-    <t>Errors if already on the final question (call /end instead). Broadcasts session:state + question:new.</t>
+    <t>Updated QuizSession (status: "in_progress")</t>
+  </si>
+  <si>
+    <t>Only valid from status "draft" and requires questions configured. Broadcasts session:state + questions:all (ALL 5 questions at once — no per-question pacing).</t>
   </si>
   <si>
     <t>/api/sessions/:id/end</t>
@@ -129,7 +111,7 @@
     <t>Updated QuizSession (status: "ended")</t>
   </si>
   <si>
-    <t>Broadcasts session:state + quiz:ended + a final leaderboard:update.</t>
+    <t>Only valid from "in_progress". Broadcasts session:state + quiz:ended + a final leaderboard:update. There is no "next question" admin control — the whole state machine is draft -&gt; in_progress -&gt; ended.</t>
   </si>
   <si>
     <t>/api/sessions/:id/leaderboard</t>
@@ -165,22 +147,22 @@
     <t>/api/sessions/:id/state?participantId=&lt;id&gt;</t>
   </si>
   <si>
-    <t>{ sessionId, title, status, currentQuestionIndex, totalQuestions, hasAnsweredCurrentQuestion: boolean|null }</t>
-  </si>
-  <si>
-    <t>participantId query param is optional; when provided, tells the client if it already answered the current question (for showing "waiting" state after refresh).</t>
+    <t>{ sessionId, title, status, totalQuestions, answeredQuestionIds: string[]|null }</t>
+  </si>
+  <si>
+    <t>participantId query param is optional; when provided (and status is not "draft"), returns which question IDs this participant has already answered — use this to resume mid-quiz after a reload.</t>
   </si>
   <si>
     <t>Questions (Public)</t>
   </si>
   <si>
-    <t>/api/questions/:sessionId/current</t>
-  </si>
-  <si>
-    <t>{ id, text, order, timeLimitSeconds, dimension, options: [{key, text}], index, totalQuestions }</t>
-  </si>
-  <si>
-    <t>No correct-answer/points info is exposed. 404 if no active question.</t>
+    <t>/api/questions/:sessionId</t>
+  </si>
+  <si>
+    <t>SanitizedQuestion[]: [{ id, text, order, timeLimitSeconds, dimension, options: [{key, text}] }]</t>
+  </si>
+  <si>
+    <t>Returns ALL questions at once (not one "current" question) — the quiz is self-paced, not admin-paced. 400 if session is still "draft" (quiz not started, questions must not leak early). No correct-answer/points info is exposed.</t>
   </si>
   <si>
     <t>Participants (Public)</t>
@@ -198,7 +180,7 @@
     <t>{ participantId: string, sessionToken: string }</t>
   </si>
   <si>
-    <t>Only works when session.status === "registration_open". Store sessionToken client-side (localStorage) — it is the bearer token for all subsequent participant calls.</t>
+    <t>Works any time the session is not yet "ended" — participants can land on the session URL directly and register whenever, no separate registration-open gate. Store sessionToken client-side (localStorage) — it is the bearer token for all subsequent participant calls.</t>
   </si>
   <si>
     <t>PATCH</t>
@@ -237,10 +219,10 @@
     <t>{ questionId: string (Mongo ObjectId), selectedKey: "A"|"B"|"C"|"D", timeTakenMs: number (&gt;= 0) }</t>
   </si>
   <si>
-    <t>Created Answer record (points are computed server-side, not trusted from client)</t>
-  </si>
-  <si>
-    <t>One answer per (participant, question) enforced by a unique index — resubmits should be treated as an error by the UI.</t>
+    <t>{ success: true } (points are computed server-side, not trusted from client)</t>
+  </si>
+  <si>
+    <t>Self-paced: any question belonging to the session can be answered in any order, as long as session.status === "in_progress". One answer per (participant, question) enforced by a unique index — resubmits return 409 Conflict.</t>
   </si>
   <si>
     <t>Analysis (Public)</t>
@@ -252,7 +234,7 @@
     <t>AnalysisReport: { participantId, sessionId, generatedAt, techScore, archetype, dimensionScores: {growthMindset, customerRelationship, strategicThinking, investmentDiscipline, digitalReadiness}, reportJson: {headline, businessSnapshot, mindsetProfile, goalRoadmap[], techRecommendation} }</t>
   </si>
   <si>
-    <t>"Analyze My Business" button. Triggers AI generation on first call; cached (idempotent) on repeat calls. Can take a few seconds — show a loading/"AI thinking" state.</t>
+    <t>"Analyze My Business" section on the results screen (shown right after quiz:ended, alongside the leaderboard). Triggers AI generation on first call; cached (idempotent) on repeat calls. Can take a few seconds — show a loading/"AI thinking" state.</t>
   </si>
   <si>
     <t>Existing AnalysisReport, or 404/null if not generated yet</t>
@@ -279,7 +261,7 @@
     <t>{ sessionId: string, participantId?: string, role: "participant" | "display" | "admin" }</t>
   </si>
   <si>
-    <t>Send immediately after connecting to the "quiz" namespace. Joins the session room (and a display sub-room if role is "display"). Server replies with session:state (and question:new if quiz is in progress).</t>
+    <t>Send immediately after connecting to the "quiz" namespace. Joins the session room (and a display sub-room if role is "display"). Server replies with session:state (and questions:all if the quiz is in_progress or already ended).</t>
   </si>
   <si>
     <t>Server → Client</t>
@@ -288,19 +270,19 @@
     <t>session:state</t>
   </si>
   <si>
-    <t>{ sessionId, title, status, currentQuestionIndex, totalQuestions, hasAnsweredCurrentQuestion }</t>
-  </si>
-  <si>
-    <t>Sent on join and on every admin state transition. Drives which screen the client shows (waiting room / question / leaderboard / final rank).</t>
-  </si>
-  <si>
-    <t>question:new</t>
-  </si>
-  <si>
-    <t>{ question: {id, text, order, timeLimitSeconds, dimension, options}, index, totalQuestions, timeLimitSeconds, serverTimestamp }</t>
-  </si>
-  <si>
-    <t>Fired when the admin starts the quiz or advances to the next question. Use serverTimestamp to sync the countdown timer across devices.</t>
+    <t>{ sessionId, title, status, totalQuestions, answeredQuestionIds }</t>
+  </si>
+  <si>
+    <t>Sent on join and on every admin state transition (start/end). Drives which screen the client shows (waiting room / quiz / results). status is one of draft | in_progress | ended — that's the whole state machine.</t>
+  </si>
+  <si>
+    <t>questions:all</t>
+  </si>
+  <si>
+    <t>{ questions: SanitizedQuestion[], totalQuestions, serverTimestamp }</t>
+  </si>
+  <si>
+    <t>Fired ONCE when the admin starts the quiz (replaces the old per-question "question:new" push — there is no next-question admin control). Contains all 5 questions; the client paces the participant through them itself and submits each via POST /api/answers as answered.</t>
   </si>
   <si>
     <t>leaderboard:update</t>
@@ -309,7 +291,7 @@
     <t>{ top: [{participantId, name, businessName?, score, rank}], totalAnswered }</t>
   </si>
   <si>
-    <t>Debounced ~1s after answers come in. top is limited to top 10 — use for the live projector display, not full rankings.</t>
+    <t>Debounced ~1s after answers come in. top is limited to top 10 — use for the live projector display, not full rankings. totalAnswered is a good proxy for "quiz progress" since there is no per-question index anymore.</t>
   </si>
   <si>
     <t>quiz:ended</t>
@@ -318,13 +300,22 @@
     <t>{}</t>
   </si>
   <si>
-    <t>Signals participants to move to their final-rank screen; followed by a final leaderboard:update.</t>
+    <t>Signals participants to go straight to the results screen (rank + leaderboard + "Analyze My Business"); followed by a final leaderboard:update.</t>
   </si>
   <si>
     <t>Base URL: all REST routes are prefixed with /api except /health.</t>
   </si>
   <si>
     <t>Socket.IO namespace: /quiz (e.g. io("https://&lt;host&gt;/quiz")).</t>
+  </si>
+  <si>
+    <t>State machine: draft -&gt; in_progress -&gt; ended. Only two admin actions: POST /api/sessions/:id/start and POST /api/sessions/:id/end. There is no "open registration" step and no "next question" step.</t>
+  </si>
+  <si>
+    <t>Registration: participants can register any time the session is not "ended" — there is no gating status to check first.</t>
+  </si>
+  <si>
+    <t>Questions: all 5 are sent to the client at once (GET /api/questions/:sessionId or the questions:all socket event) when the quiz starts. Pacing through them is entirely client-side; the server does not track or push a "current question".</t>
   </si>
   <si>
     <t>Participant auth: sessionToken returned from POST /api/participants/register, sent as "Authorization: Bearer &lt;sessionToken&gt;".</t>
@@ -731,13 +722,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="3" max="3" width="42" customWidth="1"/>
     <col min="4" max="4" width="26" customWidth="1"/>
-    <col min="5" max="7" width="55" customWidth="1"/>
+    <col min="5" max="6" width="55" customWidth="1"/>
+    <col min="7" max="7" width="60" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -883,7 +875,7 @@
         <v>20</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>33</v>
@@ -892,7 +884,7 @@
         <v>22</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>34</v>
@@ -906,7 +898,7 @@
         <v>20</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>36</v>
@@ -915,7 +907,7 @@
         <v>22</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>37</v>
@@ -949,232 +941,186 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>10</v>
+        <v>52</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>11</v>
+        <v>53</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>8</v>
+        <v>56</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>10</v>
+        <v>58</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>58</v>
+        <v>10</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>59</v>
+        <v>11</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>62</v>
+        <v>15</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>10</v>
+        <v>58</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="B17" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>72</v>
-      </c>
       <c r="D17" s="3" t="s">
-        <v>64</v>
+        <v>10</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>73</v>
+        <v>11</v>
       </c>
       <c r="F17" s="3" t="s">
         <v>74</v>
       </c>
       <c r="G17" s="3" t="s">
         <v>75</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="G19" s="3" t="s">
-        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -1191,18 +1137,19 @@
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="4" width="65" customWidth="1"/>
+    <col min="3" max="3" width="60" customWidth="1"/>
+    <col min="4" max="4" width="70" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>6</v>
@@ -1210,72 +1157,72 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>89</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -1287,7 +1234,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="110" style="4" customWidth="1"/>
@@ -1300,32 +1247,47 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>107</v>
+        <v>101</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>104</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
List past quiz sessions and surface AI failures clearly
Add GET /api/sessions (admin) so old/ended sessions stay browsable —
data was already fully session-scoped (Participant/Answer/AnalysisReport
all carry sessionId, nothing is deleted), there just wasn't a listing
endpoint yet. Also make AnthropicService throw a clear 503 instead of an
opaque 500 when both the initial and retry attempt to generate a report
fail (e.g. invalid ANTHROPIC_API_KEY), since that's what caused the
Internal server error just now.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/MACROPAGE-Quiz-API-Endpoints.xlsx
+++ b/docs/MACROPAGE-Quiz-API-Endpoints.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="108">
   <si>
     <t>Group</t>
   </si>
@@ -93,6 +93,12 @@
     <t>Creates a session; auto-seeds the 5 default questions unless autoSeedQuestions is false. Registration is open immediately — no separate open-registration step.</t>
   </si>
   <si>
+    <t>QuizSession[] — every session ever created, newest first (sorted by createdAt desc)</t>
+  </si>
+  <si>
+    <t>Quiz history / session picker. Sessions are never deleted, so past events (and their leaderboard/participants/export) stay browsable via this list + the existing per-session routes below.</t>
+  </si>
+  <si>
     <t>/api/sessions/:id/start</t>
   </si>
   <si>
@@ -120,7 +126,7 @@
     <t>LeaderboardEntry[]: { participantId, name, businessName?, score, rank }[]</t>
   </si>
   <si>
-    <t>Full ranked list (not just top N) — for admin dashboard, not the projector display.</t>
+    <t>Full ranked list (not just top N) — for admin dashboard, not the projector display. Works for past (ended) sessions too.</t>
   </si>
   <si>
     <t>/api/sessions/:id/participants</t>
@@ -129,7 +135,7 @@
     <t>Participant[] (full documents incl. onboarding fields)</t>
   </si>
   <si>
-    <t>For admin review / manual export.</t>
+    <t>For admin review / manual export. Works for past (ended) sessions too.</t>
   </si>
   <si>
     <t>/api/sessions/:id/export.csv</t>
@@ -138,7 +144,7 @@
     <t>text/csv file download (Content-Disposition: attachment)</t>
   </si>
   <si>
-    <t>Columns: Name, WhatsApp Number, Business Name, Business Category, Goal, Goal (Other), Score, Rank, Registered At.</t>
+    <t>Columns: Name, WhatsApp Number, Business Name, Business Category, Goal, Goal (Other), Score, Rank, Registered At. Works for past (ended) sessions too.</t>
   </si>
   <si>
     <t>Sessions (Public)</t>
@@ -234,7 +240,7 @@
     <t>AnalysisReport: { participantId, sessionId, generatedAt, techScore, archetype, dimensionScores: {growthMindset, customerRelationship, strategicThinking, investmentDiscipline, digitalReadiness}, reportJson: {headline, businessSnapshot, mindsetProfile, goalRoadmap[], techRecommendation} }</t>
   </si>
   <si>
-    <t>"Analyze My Business" section on the results screen (shown right after quiz:ended, alongside the leaderboard). Triggers AI generation on first call; cached (idempotent) on repeat calls. Can take a few seconds — show a loading/"AI thinking" state.</t>
+    <t>"Analyze My Business" section on the results screen (shown right after quiz:ended, alongside the leaderboard). Triggers AI generation on first call; cached (idempotent) on repeat calls. Can take a few seconds — show a loading/"AI thinking" state. Returns 503 with a clear message if the AI call fails after retrying once (e.g. bad/missing ANTHROPIC_API_KEY).</t>
   </si>
   <si>
     <t>Existing AnalysisReport, or 404/null if not generated yet</t>
@@ -310,6 +316,9 @@
   </si>
   <si>
     <t>State machine: draft -&gt; in_progress -&gt; ended. Only two admin actions: POST /api/sessions/:id/start and POST /api/sessions/:id/end. There is no "open registration" step and no "next question" step.</t>
+  </si>
+  <si>
+    <t>Session history: sessions are never deleted. GET /api/sessions lists all of them (newest first) so past events stay browsable via the existing per-session leaderboard/participants/export routes.</t>
   </si>
   <si>
     <t>Registration: participants can register any time the session is not "ended" — there is no gating status to check first.</t>
@@ -722,7 +731,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -829,22 +838,22 @@
         <v>20</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>22</v>
       </c>
       <c r="E5" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5" s="3" t="s">
         <v>27</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -855,19 +864,19 @@
         <v>15</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>22</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F6" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G6" s="3" t="s">
         <v>31</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -875,22 +884,22 @@
         <v>20</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>22</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="F7" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G7" s="3" t="s">
         <v>34</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -901,7 +910,7 @@
         <v>8</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>22</v>
@@ -910,10 +919,10 @@
         <v>11</v>
       </c>
       <c r="F8" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="G8" s="3" t="s">
         <v>37</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -924,7 +933,7 @@
         <v>8</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>22</v>
@@ -933,44 +942,44 @@
         <v>11</v>
       </c>
       <c r="F9" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="G9" s="3" t="s">
         <v>40</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>10</v>
@@ -979,148 +988,171 @@
         <v>11</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F12" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B12" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C12" s="3" t="s">
+      <c r="G12" s="3" t="s">
         <v>51</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B13" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="F13" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="G13" s="3" t="s">
         <v>57</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>8</v>
+        <v>58</v>
       </c>
       <c r="C14" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="F14" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="D14" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F14" s="3" t="s">
+      <c r="G14" s="3" t="s">
         <v>63</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F15" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="B15" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C15" s="3" t="s">
+      <c r="G15" s="3" t="s">
         <v>66</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="G15" s="3" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>15</v>
       </c>
       <c r="C16" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="G16" s="3" t="s">
         <v>71</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="F17" s="3" t="s">
         <v>74</v>
       </c>
       <c r="G17" s="3" t="s">
         <v>75</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -1143,13 +1175,13 @@
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>6</v>
@@ -1157,72 +1189,72 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -1234,7 +1266,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="110" style="4" customWidth="1"/>
@@ -1247,47 +1279,52 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>104</v>
+        <v>106</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>107</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Re-add open-registration as an explicit admin step
Restores the registration_open state that was dropped in the earlier
flow simplification: draft -> registration_open -> in_progress -> ended.
Registration (POST /api/participants/register) is now only accepted
while status is exactly "registration_open", via the new
POST /api/sessions/:id/open-registration admin action. Start now
transitions from registration_open instead of draft. Question fetching
(GET /api/questions/:sessionId) is likewise blocked until in_progress,
not just during draft.

Updated README and the frontend build prompt/API spreadsheet to match.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/MACROPAGE-Quiz-API-Endpoints.xlsx
+++ b/docs/MACROPAGE-Quiz-API-Endpoints.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="124">
   <si>
     <t>Group</t>
   </si>
@@ -132,7 +132,7 @@
     <t>SanitizedQuestion[]: [{ id, text, order, timeLimitSeconds, type: "mindset"|"trivia", dimension?, options: [{key, text}] }]</t>
   </si>
   <si>
-    <t>THIS PARTICIPANT'S OWN question set, not a shared session list: 5 mindset questions (one randomly sampled per dimension from the bank, assigned on first call and persisted on Participant.assignedQuestionIds — same set returned on every later call/reload) + the session's shared trivia questions appended after. 400 if session is still "draft". No correct-answer/points info exposed.</t>
+    <t>THIS PARTICIPANT'S OWN question set, not a shared session list: 5 mindset questions (one randomly sampled per dimension from the bank, assigned on first call and persisted on Participant.assignedQuestionIds — same set returned on every later call/reload) + the session's shared trivia questions appended after. 400 unless status is "in_progress" or "ended" (i.e. still blocked during "draft" and "registration_open"). No correct-answer/points info exposed.</t>
   </si>
   <si>
     <t>Sessions (Admin)</t>
@@ -147,7 +147,7 @@
     <t>QuizSession document (_id, status: "draft", questionIds: [] — trivia only)</t>
   </si>
   <si>
-    <t>Creates a session. Mindset questions are NOT configured here — they are assigned per participant, not per session. Optionally appends trivia: triviaQuestionIds is an explicit, ordered pick (takes priority if both are sent); triviaCount randomly samples that many from the trivia bank via $sample. Registration is open immediately — no separate open-registration step.</t>
+    <t>Creates a session. Mindset questions are NOT configured here — they are assigned per participant, not per session. Optionally appends trivia: triviaQuestionIds is an explicit, ordered pick (takes priority if both are sent); triviaCount randomly samples that many from the trivia bank via $sample. Registration is NOT open yet — admin must call open-registration below.</t>
   </si>
   <si>
     <t>QuizSession[] — every session ever created, newest first (sorted by createdAt desc)</t>
@@ -156,13 +156,22 @@
     <t>Quiz history / session picker. Sessions are never deleted, so past events (and their leaderboard/participants/export) stay browsable via this list + the existing per-session routes below.</t>
   </si>
   <si>
+    <t>/api/sessions/:id/open-registration</t>
+  </si>
+  <si>
+    <t>Updated QuizSession (status: "registration_open")</t>
+  </si>
+  <si>
+    <t>Only valid from status "draft". Once open, participants can call POST /api/participants/register — it 400s at every other status.</t>
+  </si>
+  <si>
     <t>/api/sessions/:id/start</t>
   </si>
   <si>
     <t>Updated QuizSession (status: "in_progress")</t>
   </si>
   <si>
-    <t>Only valid from status "draft". 400s if the global mindset bank is empty (call POST /api/questions/mindset/seed first) — this replaced the old "session has no questions configured" check, since mindset is no longer session-scoped.</t>
+    <t>Only valid from status "registration_open". 400s if the global mindset bank is empty (call POST /api/questions/mindset/seed first) — this replaced the old "session has no questions configured" check, since mindset is no longer session-scoped.</t>
   </si>
   <si>
     <t>/api/sessions/:id/end</t>
@@ -171,7 +180,7 @@
     <t>Updated QuizSession (status: "ended")</t>
   </si>
   <si>
-    <t>Only valid from "in_progress". Broadcasts session:state + quiz:ended + a final leaderboard:update. There is no "next question" admin control — the whole state machine is draft -&gt; in_progress -&gt; ended.</t>
+    <t>Only valid from "in_progress". Broadcasts session:state + quiz:ended + a final leaderboard:update. There is no "next question" admin control — the full state machine is draft -&gt; registration_open -&gt; in_progress -&gt; ended.</t>
   </si>
   <si>
     <t>/api/sessions/:id/leaderboard</t>
@@ -228,7 +237,7 @@
     <t>{ participantId: string, sessionToken: string }</t>
   </si>
   <si>
-    <t>Works any time the session is not yet "ended" — participants can land on the session URL directly and register whenever, no separate registration-open gate. Store sessionToken client-side (localStorage) — it is the bearer token for all subsequent participant calls.</t>
+    <t>Only accepted while session.status === "registration_open" (admin must call POST /api/sessions/:id/open-registration first) — 400 at any other status. Store sessionToken client-side (localStorage) — it is the bearer token for all subsequent participant calls.</t>
   </si>
   <si>
     <t>PATCH</t>
@@ -345,7 +354,7 @@
     <t>Socket.IO namespace: /quiz (e.g. io("https://&lt;host&gt;/quiz")).</t>
   </si>
   <si>
-    <t>State machine: draft -&gt; in_progress -&gt; ended. Only two admin actions: POST /api/sessions/:id/start and POST /api/sessions/:id/end. There is no "open registration" step and no "next question" step.</t>
+    <t>State machine: draft -&gt; registration_open -&gt; in_progress -&gt; ended, strictly linear. Three admin actions drive it: POST /api/sessions/:id/open-registration, POST /api/sessions/:id/start, POST /api/sessions/:id/end. There is no "next question" step.</t>
   </si>
   <si>
     <t>PERSONALIZED QUESTIONS: each participant gets their own random pick of 1 mindset question per dimension (5 total, from a 15-question bank with 3 variants per dimension), assigned on their first GET /api/questions/:sessionId call and persisted on Participant.assignedQuestionIds — the same set is returned on every later call. Different participants very likely see different specific wording for the same dimension. This guarantees full dimension coverage per participant, so the AI analysis always has complete data.</t>
@@ -357,7 +366,7 @@
     <t>Session history: sessions are never deleted. GET /api/sessions lists all of them (newest first) so past events stay browsable via the existing per-session leaderboard/participants/export routes.</t>
   </si>
   <si>
-    <t>Registration: participants can register any time the session is not "ended" — there is no gating status to check first.</t>
+    <t>Registration: only accepted while session.status === "registration_open" — the admin must explicitly open it via POST /api/sessions/:id/open-registration before the QR/join URL will accept POST /api/participants/register.</t>
   </si>
   <si>
     <t>No socket event carries question content. Once session:state.status becomes in_progress, the client must call GET /api/questions/:sessionId (bearer sessionToken) to fetch its own set — this was previously a broadcast "questions:all" socket event, removed because content is now personalized per participant and cannot be broadcast identically to a room.</t>
@@ -770,7 +779,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -1061,7 +1070,7 @@
         <v>40</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>53</v>
@@ -1070,7 +1079,7 @@
         <v>22</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="F13" s="3" t="s">
         <v>54</v>
@@ -1127,88 +1136,88 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F16" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="G16" s="3" t="s">
         <v>64</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="B17" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C17" s="3" t="s">
+      <c r="D17" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F17" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="G17" s="3" t="s">
         <v>68</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="G17" s="3" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B18" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="E18" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="F18" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D18" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="E18" s="3" t="s">
+      <c r="G18" s="3" t="s">
         <v>74</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>8</v>
+        <v>75</v>
       </c>
       <c r="C19" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E19" s="3" t="s">
         <v>77</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>11</v>
       </c>
       <c r="F19" s="3" t="s">
         <v>78</v>
@@ -1219,71 +1228,94 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="B20" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C20" s="3" t="s">
+      <c r="D20" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F20" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="D20" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="E20" s="3" t="s">
+      <c r="G20" s="3" t="s">
         <v>82</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>15</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="D21" s="3" t="s">
         <v>37</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>23</v>
+        <v>85</v>
       </c>
       <c r="F21" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="G21" s="3" t="s">
         <v>87</v>
-      </c>
-      <c r="G21" s="3" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B22" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B23" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C22" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="D22" s="3" t="s">
+      <c r="C23" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="D23" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="E22" s="3" t="s">
+      <c r="E23" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F22" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="G22" s="3" t="s">
-        <v>90</v>
+      <c r="F23" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -1306,13 +1338,13 @@
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>6</v>
@@ -1320,58 +1352,58 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>
@@ -1396,67 +1428,67 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>

</xml_diff>